<commit_message>
Harden eval scorer + add real-quote drop-in path (Codex review #2 & #4)
- Strict line-item match: amount ±1% AND unit match AND qty ±2% (was amount-only,
  flagged 'gameable'). Still 100% recall on the synthetic corpus -> defensible.
- EVIDENCE.md states the strict scoring methodology explicitly + that synthetic is
  an upper bound; real estimator-labeled benchmark is the next step.
- demo/real/ drop-in path for real anonymized estimator-labeled quotes (Codex's
  #1 unlock; needs real data, not fabrication).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/leveling_drywall.xlsx
+++ b/demo/leveling_drywall.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -569,7 +569,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Drywall</t>
+          <t>Drywall &amp; Framing</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -714,7 +714,7 @@
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>High scaffolding</t>
+          <t>Scaffolding over 10ft</t>
         </is>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -723,11 +723,7 @@
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr"/>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>EXCL (p1)</t>
-        </is>
-      </c>
+      <c r="D14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -763,7 +759,11 @@
           <t>EXCL (p1)</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr"/>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>EXCL (p1)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -814,7 +814,7 @@
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>Demolition</t>
+          <t>Demolition of existing walls/ceilings</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
@@ -823,12 +823,16 @@
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr"/>
-      <c r="D21" s="7" t="inlineStr"/>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Waste removal (beyond final cleaning)</t>
+          <t>Protection of adjacent finishes/work</t>
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr">
@@ -842,7 +846,7 @@
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>Protection of adjacent work</t>
+          <t>Daily debris removal/waste management</t>
         </is>
       </c>
       <c r="B23" s="13" t="inlineStr">
@@ -850,17 +854,13 @@
           <t>⚠</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
+      <c r="C23" s="7" t="inlineStr"/>
       <c r="D23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Painting/Priming</t>
+          <t>Blocking for wall-mounted items (e.g., cabinets, fixtures)</t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
@@ -878,21 +878,21 @@
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>Fire caulking at penetrations</t>
-        </is>
-      </c>
-      <c r="B25" s="13" t="inlineStr">
+          <t>Demolition/Patching</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr"/>
+      <c r="C25" s="13" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
       <c r="D25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>Waste removal (daily/rough cleanup)</t>
+          <t>Corner Bead/Trim</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr"/>
@@ -906,7 +906,7 @@
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>Demolition or patching of existing walls</t>
+          <t>Blocking/Backing</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr"/>
@@ -920,25 +920,29 @@
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>Demolition of existing drywall</t>
+          <t>Sound Caulking</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr"/>
-      <c r="C28" s="7" t="inlineStr"/>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="C28" s="13" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
       </c>
+      <c r="D28" s="7" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>Sound caulking</t>
+          <t>Access Panels</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr"/>
-      <c r="C29" s="7" t="inlineStr"/>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
           <t>⚠</t>
@@ -948,12 +952,54 @@
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>Protection of adjacent finishes</t>
+          <t>Protection of adjacent surfaces</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr"/>
       <c r="C30" s="7" t="inlineStr"/>
       <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Waste removal (beyond final cleaning)</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr"/>
+      <c r="C31" s="7" t="inlineStr"/>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Specific finish levels (e.g., Level 5 finish)</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr"/>
+      <c r="C32" s="7" t="inlineStr"/>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Acoustic sealant</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr"/>
+      <c r="C33" s="7" t="inlineStr"/>
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
@@ -1603,28 +1649,28 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>(p1) Fire-stopping EXCLUDED.</t>
+          <t>(p1) 1. Fire-stopping EXCLUDED.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>(p1) Insulation EXCLUDED.</t>
+          <t>(p1) 2. Insulation EXCLUDED.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>(p1) Scaffolding EXCLUDED.</t>
+          <t>(p1) 3. Scaffolding EXCLUDED.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>(p1) Final cleaning EXCLUDED.</t>
+          <t>(p1) 4. Final cleaning EXCLUDED.</t>
         </is>
       </c>
     </row>

</xml_diff>